<commit_message>
update training data with 250+ more entries
</commit_message>
<xml_diff>
--- a/data/raw/test2026-06-13/lakewood_spreadsheet1_v4.xlsx
+++ b/data/raw/test2026-06-13/lakewood_spreadsheet1_v4.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="175">
   <si>
     <t>intersection</t>
   </si>
@@ -25,28 +25,85 @@
     <t>notes</t>
   </si>
   <si>
+    <t>evans-wadsworth</t>
+  </si>
+  <si>
+    <t>Circle K</t>
+  </si>
+  <si>
+    <t>storefront_main</t>
+  </si>
+  <si>
+    <t>Orion's Center</t>
+  </si>
+  <si>
+    <t>storefront_accessory</t>
+  </si>
+  <si>
+    <t>Popeyes</t>
+  </si>
+  <si>
+    <t>girton-wadsworth</t>
+  </si>
+  <si>
+    <t>Girton Ave</t>
+  </si>
+  <si>
+    <t>street_sign</t>
+  </si>
+  <si>
+    <t>Common Spirit Emergency and Urgent Care</t>
+  </si>
+  <si>
+    <t>Natural Grocers</t>
+  </si>
+  <si>
+    <t>yale-wadsworth</t>
+  </si>
+  <si>
+    <t>La-Z-Boy</t>
+  </si>
+  <si>
+    <t>Stanley Steemer</t>
+  </si>
+  <si>
+    <t>advertisement</t>
+  </si>
+  <si>
+    <t>Wild Birds Unlimited</t>
+  </si>
+  <si>
+    <t>alameda-wadsworth</t>
+  </si>
+  <si>
+    <t>1st-wadsworth</t>
+  </si>
+  <si>
+    <t>2nd-union</t>
+  </si>
+  <si>
+    <t>bowles-coalmine</t>
+  </si>
+  <si>
+    <t>colfax-simms</t>
+  </si>
+  <si>
+    <t>colfax-kipling</t>
+  </si>
+  <si>
     <t>morrison-wadsworth</t>
   </si>
   <si>
     <t>innovage all-inclusive care for the elderly - age independently in your own home</t>
   </si>
   <si>
-    <t>advertisement</t>
-  </si>
-  <si>
     <t>innovage innovage</t>
   </si>
   <si>
     <t>morrison rd</t>
   </si>
   <si>
-    <t>street_sign</t>
-  </si>
-  <si>
     <t>alpine dental arts</t>
-  </si>
-  <si>
-    <t>storefront_main</t>
   </si>
   <si>
     <t>venture resources inc</t>
@@ -125,30 +182,6 @@
     <t>access-a-ride</t>
   </si>
   <si>
-    <t>girton-wadsworth</t>
-  </si>
-  <si>
-    <t>Girton Ave</t>
-  </si>
-  <si>
-    <t>Common Spirit Emergency and Urgent Care</t>
-  </si>
-  <si>
-    <t>Natural Grocers</t>
-  </si>
-  <si>
-    <t>yale-wadsworth</t>
-  </si>
-  <si>
-    <t>La-Z-Boy</t>
-  </si>
-  <si>
-    <t>Stanley Steemer</t>
-  </si>
-  <si>
-    <t>Wild Birds Unlimited</t>
-  </si>
-  <si>
     <t>No Right Turn on Red</t>
   </si>
   <si>
@@ -161,19 +194,214 @@
     <t>Touchstone Dental and Implants</t>
   </si>
   <si>
-    <t>evans-wadsworth</t>
-  </si>
-  <si>
-    <t>Circle K</t>
-  </si>
-  <si>
-    <t>Orion's Center</t>
-  </si>
-  <si>
-    <t>storefront_accessory</t>
-  </si>
-  <si>
-    <t>Popeyes</t>
+    <t>mississippi-sheridan</t>
+  </si>
+  <si>
+    <t>&lt;- mississippi ave</t>
+  </si>
+  <si>
+    <t>Denver Morrison Rd -&gt;</t>
+  </si>
+  <si>
+    <t>welcome to westwood denver</t>
+  </si>
+  <si>
+    <t>other_sign</t>
+  </si>
+  <si>
+    <t>7 eleven first cash pawn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 eleven 7 eleven </t>
+  </si>
+  <si>
+    <t>7 eleeven</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">no fuss foundation repair colorado structural repair colorado's bes rated local foundation repair company google us! </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>coloradostructuralrepair.com</t>
+    </r>
+  </si>
+  <si>
+    <t>marlboro</t>
+  </si>
+  <si>
+    <t>fast cash pawn &amp; gold center</t>
+  </si>
+  <si>
+    <t>fast cash pawn &amp; jewlery</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>entrance fast cash</t>
+  </si>
+  <si>
+    <t>pawn &amp; jewelry gold diamonds tv's tools cameras guns</t>
+  </si>
+  <si>
+    <t>fast cash pawn &amp; gold center 7 eleven</t>
+  </si>
+  <si>
+    <t>lot_sign</t>
+  </si>
+  <si>
+    <t>llantes tires</t>
+  </si>
+  <si>
+    <t>quiktrip</t>
+  </si>
+  <si>
+    <t>QT QT QT</t>
+  </si>
+  <si>
+    <t>first cash pawn</t>
+  </si>
+  <si>
+    <t>11 aurora met ctr</t>
+  </si>
+  <si>
+    <t>bus</t>
+  </si>
+  <si>
+    <t>phone repair and more</t>
+  </si>
+  <si>
+    <t>speed limit 35</t>
+  </si>
+  <si>
+    <t>city of lakewood adopt a street joyful journeys community enrichment jeffco</t>
+  </si>
+  <si>
+    <t>tamales moreno mexican food</t>
+  </si>
+  <si>
+    <t>tamale kitchen</t>
+  </si>
+  <si>
+    <t>tamale kitchen mexican food</t>
+  </si>
+  <si>
+    <t>tamale kitchen burritos tamales tacos green chile beans empanaditas rice chicharones</t>
+  </si>
+  <si>
+    <t>harts corner</t>
+  </si>
+  <si>
+    <t>tamale kitchen plaza centro de nutricion summer spa truth barbershop tamale kitchen mexican restaurant tamales</t>
+  </si>
+  <si>
+    <t>mexican haburger chili cheese fires chile rellenos</t>
+  </si>
+  <si>
+    <t>truck</t>
+  </si>
+  <si>
+    <t>uhaul center open 7 days uhaul center</t>
+  </si>
+  <si>
+    <t>19.95 in-town plus mileage/fees drive now rent your phone truck share 24/7 u-haul app u-haul truck share 24/7</t>
+  </si>
+  <si>
+    <t>19.95 in-town plus mileage/fees drive now rent your phone truck share 24/7 u-haul app u-haul truck share 24/8</t>
+  </si>
+  <si>
+    <t>19.95 in-town plus mileage/fees drive now rent your phone truck share 24/7 u-haul app u-haul truck share 24/9</t>
+  </si>
+  <si>
+    <t>in-town special! 19.95</t>
+  </si>
+  <si>
+    <t>www.uhaul.com</t>
+  </si>
+  <si>
+    <t>auto hail repair</t>
+  </si>
+  <si>
+    <t>u-haul right equipment / lowest cost fuel saver chassie skirts</t>
+  </si>
+  <si>
+    <t>your morning me-time M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpr for your roof colorado </t>
+  </si>
+  <si>
+    <t>fired cannabis</t>
+  </si>
+  <si>
+    <t>reserved</t>
+  </si>
+  <si>
+    <t>louisiana ave next signal</t>
+  </si>
+  <si>
+    <t>flamingos night club</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">frank AZAR truck crash? </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>fdazar.com</t>
+    </r>
+  </si>
+  <si>
+    <t>últimonivel</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">now enrolling senior social club former young adult day center </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>www.seniorluv.net</t>
+    </r>
+  </si>
+  <si>
+    <t>la pachanga nightclub</t>
+  </si>
+  <si>
+    <t>left 2 lanes must turn left</t>
+  </si>
+  <si>
+    <t>tacos</t>
+  </si>
+  <si>
+    <t>boogie down su n menuro o &amp; mimosas s mo n poo l tou any 5 pm tue tacos ing o 6 pm we d. 530 any shots</t>
+  </si>
+  <si>
+    <t>$18 bud light buckets</t>
+  </si>
+  <si>
+    <t>bud light bud light bud light bud light bud light bud light bud light</t>
+  </si>
+  <si>
+    <t>official Denver Sponsor Michelob Ultra Denver Denver Denver</t>
   </si>
   <si>
     <t>jewell-garrison</t>
@@ -188,22 +416,196 @@
     <t>Coca Cola</t>
   </si>
   <si>
-    <t>alameda-wadsworth</t>
-  </si>
-  <si>
-    <t>1st-wadsworth</t>
-  </si>
-  <si>
-    <t>2nd-union</t>
-  </si>
-  <si>
-    <t>bowles-coalmine</t>
-  </si>
-  <si>
-    <t>colfax-simms</t>
-  </si>
-  <si>
-    <t>colfax-kipling</t>
+    <t>jiu-jitsu kickboxing</t>
+  </si>
+  <si>
+    <t>flolife BJJ+</t>
+  </si>
+  <si>
+    <t>blackjack pizza &amp; salads $2.99 lunch special</t>
+  </si>
+  <si>
+    <t xml:space="preserve">now hiring delivery divers wings calzones desserts handcrafted crunchy crust. smothered in cheese. </t>
+  </si>
+  <si>
+    <t>blackjackpizza.com</t>
+  </si>
+  <si>
+    <t>desserts salads</t>
+  </si>
+  <si>
+    <t>ahead</t>
+  </si>
+  <si>
+    <t>private parking</t>
+  </si>
+  <si>
+    <t>donut burst coffee &amp; donuts</t>
+  </si>
+  <si>
+    <t>13 fresh donutes 9.99</t>
+  </si>
+  <si>
+    <t>ice cream $1.39</t>
+  </si>
+  <si>
+    <t>jewell park city of lakewood 1852 S Garrison st</t>
+  </si>
+  <si>
+    <t>yield here to</t>
+  </si>
+  <si>
+    <t>city of lakewood adopt a gulch no motorized vehicles</t>
+  </si>
+  <si>
+    <t>unlawful to cross into immediate path of vehicle</t>
+  </si>
+  <si>
+    <t>right lane only</t>
+  </si>
+  <si>
+    <t>city of lakwood</t>
+  </si>
+  <si>
+    <t>begin right turn lane yield to bikes</t>
+  </si>
+  <si>
+    <t>slammin chicken</t>
+  </si>
+  <si>
+    <t>tokyo hibachi express</t>
+  </si>
+  <si>
+    <t>bike lane</t>
+  </si>
+  <si>
+    <t>blackjack pizza $9.99 anytime! blackjack pizza lord &amp; fuchs properties llp lakewood liquors the prophet salon jiu-jitsu &amp; kickboxing</t>
+  </si>
+  <si>
+    <t>Garrison St 9200 W</t>
+  </si>
+  <si>
+    <t>U-Haul Moving &amp; Storage open 7 days u-box move + store we ship anywhere</t>
+  </si>
+  <si>
+    <t>custom hitches u-haul center the box store</t>
+  </si>
+  <si>
+    <t>uhaul uhaul</t>
+  </si>
+  <si>
+    <t>u-haul</t>
+  </si>
+  <si>
+    <t>scouts meet here boy scouts Weds. 7PM</t>
+  </si>
+  <si>
+    <t>our saviour's church</t>
+  </si>
+  <si>
+    <t>propane fast fill fast pay at the pump new! u-haul $4.10 gal</t>
+  </si>
+  <si>
+    <t>big sky burgers</t>
+  </si>
+  <si>
+    <t>burgers fries shakes</t>
+  </si>
+  <si>
+    <t>fried rice ramen</t>
+  </si>
+  <si>
+    <t>woodlake center garramone's pizza italian restaurant gourmet meats barney's barbershop corky's bookkeeping aspen environmental home cleaners of america westwood travel skin care native zen massage health touch massage dance family clinic pet grooming garrison st. stylists tea shop &amp; studio</t>
+  </si>
+  <si>
+    <t>exit only</t>
+  </si>
+  <si>
+    <t>unauthorized or improperly parked vehicles will be towed and impounded at vehicle owners expense maxx auto recovery, inc.</t>
+  </si>
+  <si>
+    <t>barney's arber shop</t>
+  </si>
+  <si>
+    <t>no parking</t>
+  </si>
+  <si>
+    <t>barbershoop</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">celtic steps </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>celticsteps.org</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> first class free please use the back entrance</t>
+    </r>
+  </si>
+  <si>
+    <t>lakewood health clinic</t>
+  </si>
+  <si>
+    <t>acupuncture &amp; eastern healing</t>
+  </si>
+  <si>
+    <t>corky's bookkeeping &amp; taxd income tax preparation</t>
+  </si>
+  <si>
+    <t>foot massage foot+body 1hr $39.99</t>
+  </si>
+  <si>
+    <t>massage therapy</t>
+  </si>
+  <si>
+    <t>hair styling salon</t>
+  </si>
+  <si>
+    <t>garrison st stylists</t>
+  </si>
+  <si>
+    <t>haircare</t>
+  </si>
+  <si>
+    <t>the collective botiques connect create</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">the collective welcomes poetic tea open 9--1 thu, fri &amp; sat &amp; by reservation for speacila events poetictea.com </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>collectivebotiques.com</t>
+    </r>
+  </si>
+  <si>
+    <t>liquor</t>
+  </si>
+  <si>
+    <t>budweiser</t>
+  </si>
+  <si>
+    <t>corona</t>
+  </si>
+  <si>
+    <t>mikes hard lemonade cold hard refreshing miller light bud light bud light $19.99 24 pack cans bud light coors light fat tire newcastle brown ale la vida más finacorona $16.99 12-pack bottles drive through open $18.99</t>
+  </si>
+  <si>
+    <t>10 minute liquor store packing only</t>
+  </si>
+  <si>
+    <t>lakewood liquors</t>
   </si>
 </sst>
 </file>
@@ -233,11 +635,12 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
-      <color rgb="FF0A53A8"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <color theme="1"/>
+      <u/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -279,13 +682,13 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -527,7 +930,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="15.0" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -542,11 +945,11 @@
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -554,95 +957,63 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="B5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="B6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="B7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="B8" s="4"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>6</v>
@@ -650,21 +1021,21 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>6</v>
@@ -672,277 +1043,235 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="6"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="6"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="6"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="6"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>27</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B19" s="4"/>
       <c r="C19" s="6"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>24</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="6"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>29</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B21" s="4"/>
       <c r="C21" s="6"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>30</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B22" s="4"/>
       <c r="C22" s="6"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>6</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="6"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="6"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>6</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="6"/>
     </row>
     <row r="26">
-      <c r="A26" s="6"/>
+      <c r="A26" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="B26" s="4"/>
       <c r="C26" s="6"/>
     </row>
     <row r="27">
-      <c r="A27" s="6"/>
+      <c r="A27" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="B27" s="4"/>
       <c r="C27" s="6"/>
     </row>
     <row r="28">
-      <c r="A28" s="3"/>
+      <c r="A28" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="B28" s="4"/>
-      <c r="C28" s="3"/>
+      <c r="C28" s="6"/>
     </row>
     <row r="29">
-      <c r="A29" s="3"/>
+      <c r="A29" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="B29" s="4"/>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30">
+      <c r="C29" s="6"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1">
       <c r="A30" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>9</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="6"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="6"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="6"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>40</v>
+        <v>26</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>49</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>6</v>
@@ -950,785 +1279,1581 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B45" s="4"/>
-      <c r="C45" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B46" s="4"/>
-      <c r="C46" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B48" s="4"/>
-      <c r="C48" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B49" s="4"/>
-      <c r="C49" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="C50" s="6"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B51" s="4"/>
-      <c r="C51" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="C52" s="6"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B53" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="C53" s="6"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B54" s="4"/>
-      <c r="C54" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55" s="4"/>
-      <c r="C55" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" ht="15.0" customHeight="1">
+      <c r="A57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" ht="15.0" customHeight="1">
+      <c r="A58" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" ht="15.0" customHeight="1">
+      <c r="A59" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B56" s="4"/>
-      <c r="C56" s="6"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B57" s="4"/>
-      <c r="C57" s="6"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="4"/>
-      <c r="C58" s="6"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59" s="4"/>
-      <c r="C59" s="6"/>
-    </row>
-    <row r="60" ht="16.5" customHeight="1">
-      <c r="A60" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B60" s="4"/>
-      <c r="C60" s="6"/>
+      <c r="C60" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B61" s="4"/>
-      <c r="C61" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="4"/>
-      <c r="C62" s="6"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="6"/>
-      <c r="B63" s="4"/>
-      <c r="C63" s="6"/>
+      <c r="C63" s="3" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="6"/>
-      <c r="B64" s="4"/>
-      <c r="C64" s="6"/>
+      <c r="A64" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="6"/>
-      <c r="B65" s="4"/>
-      <c r="C65" s="6"/>
+      <c r="A65" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="6"/>
-      <c r="B66" s="4"/>
-      <c r="C66" s="6"/>
+      <c r="A66" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="6"/>
-      <c r="B67" s="4"/>
-      <c r="C67" s="6"/>
+      <c r="A67" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="6"/>
-      <c r="B68" s="4"/>
-      <c r="C68" s="6"/>
+      <c r="A68" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="6"/>
-      <c r="B69" s="4"/>
-      <c r="C69" s="6"/>
+      <c r="A69" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="6"/>
-      <c r="B70" s="4"/>
-      <c r="C70" s="6"/>
+      <c r="A70" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="6"/>
-      <c r="B71" s="4"/>
-      <c r="C71" s="6"/>
+      <c r="A71" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="6"/>
-      <c r="B72" s="4"/>
-      <c r="C72" s="6"/>
+      <c r="A72" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="6"/>
-      <c r="B73" s="4"/>
-      <c r="C73" s="6"/>
+      <c r="A73" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="6"/>
-      <c r="B74" s="4"/>
-      <c r="C74" s="6"/>
+      <c r="A74" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="6"/>
-      <c r="B75" s="4"/>
-      <c r="C75" s="6"/>
+      <c r="A75" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="6"/>
-      <c r="B76" s="4"/>
-      <c r="C76" s="6"/>
+      <c r="A76" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="6"/>
-      <c r="B77" s="4"/>
-      <c r="C77" s="6"/>
+      <c r="A77" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="6"/>
-      <c r="B78" s="4"/>
-      <c r="C78" s="6"/>
+      <c r="A78" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="6"/>
-      <c r="B79" s="4"/>
-      <c r="C79" s="6"/>
+      <c r="A79" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="6"/>
-      <c r="B80" s="4"/>
-      <c r="C80" s="6"/>
+      <c r="A80" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="6"/>
-      <c r="B81" s="4"/>
-      <c r="C81" s="6"/>
+      <c r="A81" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="6"/>
-      <c r="B82" s="4"/>
-      <c r="C82" s="6"/>
+      <c r="A82" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="6"/>
-      <c r="B83" s="4"/>
-      <c r="C83" s="6"/>
+      <c r="A83" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="6"/>
-      <c r="B84" s="4"/>
-      <c r="C84" s="6"/>
+      <c r="A84" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="6"/>
-      <c r="B85" s="4"/>
-      <c r="C85" s="6"/>
+      <c r="A85" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="6"/>
-      <c r="B86" s="4"/>
-      <c r="C86" s="6"/>
+      <c r="A86" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="6"/>
-      <c r="B87" s="4"/>
-      <c r="C87" s="6"/>
+      <c r="A87" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="6"/>
-      <c r="B88" s="4"/>
-      <c r="C88" s="6"/>
+      <c r="A88" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="6"/>
-      <c r="B89" s="4"/>
-      <c r="C89" s="6"/>
+      <c r="A89" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="6"/>
-      <c r="B90" s="4"/>
-      <c r="C90" s="6"/>
+      <c r="A90" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="6"/>
-      <c r="B91" s="4"/>
-      <c r="C91" s="6"/>
+      <c r="A91" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="6"/>
-      <c r="B92" s="4"/>
-      <c r="C92" s="6"/>
+      <c r="A92" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="6"/>
-      <c r="B93" s="4"/>
-      <c r="C93" s="6"/>
+      <c r="A93" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="6"/>
-      <c r="B94" s="4"/>
-      <c r="C94" s="6"/>
+      <c r="A94" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="6"/>
-      <c r="B95" s="4"/>
-      <c r="C95" s="6"/>
+      <c r="A95" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="6"/>
-      <c r="B96" s="4"/>
-      <c r="C96" s="6"/>
+      <c r="A96" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="6"/>
-      <c r="B97" s="4"/>
-      <c r="C97" s="6"/>
+      <c r="A97" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="6"/>
-      <c r="B98" s="4"/>
-      <c r="C98" s="6"/>
+      <c r="A98" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="6"/>
-      <c r="B99" s="4"/>
-      <c r="C99" s="6"/>
+      <c r="A99" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="6"/>
-      <c r="B100" s="4"/>
-      <c r="C100" s="6"/>
+      <c r="A100" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="6"/>
-      <c r="B101" s="4"/>
-      <c r="C101" s="6"/>
+      <c r="A101" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="6"/>
-      <c r="B102" s="4"/>
-      <c r="C102" s="6"/>
+      <c r="A102" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="6"/>
-      <c r="B103" s="4"/>
-      <c r="C103" s="6"/>
+      <c r="A103" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="6"/>
-      <c r="B104" s="4"/>
-      <c r="C104" s="6"/>
+      <c r="A104" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="6"/>
-      <c r="B105" s="4"/>
-      <c r="C105" s="6"/>
+      <c r="A105" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="6"/>
-      <c r="B106" s="4"/>
-      <c r="C106" s="6"/>
+      <c r="A106" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="6"/>
-      <c r="B107" s="4"/>
-      <c r="C107" s="6"/>
+      <c r="A107" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="6"/>
-      <c r="B108" s="4"/>
-      <c r="C108" s="6"/>
+      <c r="A108" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="6"/>
-      <c r="B109" s="4"/>
-      <c r="C109" s="6"/>
+      <c r="A109" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="6"/>
-      <c r="B110" s="4"/>
-      <c r="C110" s="6"/>
+      <c r="A110" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="8"/>
-      <c r="B111" s="9"/>
-      <c r="C111" s="10"/>
+      <c r="A111" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B111" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C111" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="8"/>
-      <c r="B112" s="9"/>
-      <c r="C112" s="10"/>
+      <c r="A112" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="8"/>
-      <c r="B113" s="9"/>
-      <c r="C113" s="10"/>
+      <c r="A113" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B113" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C113" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="8"/>
-      <c r="B114" s="9"/>
-      <c r="C114" s="10"/>
+      <c r="A114" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="8"/>
-      <c r="B115" s="9"/>
-      <c r="C115" s="10"/>
+      <c r="A115" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C115" s="9" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="8"/>
-      <c r="B116" s="9"/>
-      <c r="C116" s="10"/>
+      <c r="A116" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C116" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="8"/>
-      <c r="B117" s="9"/>
-      <c r="C117" s="10"/>
+      <c r="A117" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C117" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="8"/>
-      <c r="B118" s="9"/>
-      <c r="C118" s="10"/>
+      <c r="A118" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C118" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="8"/>
-      <c r="B119" s="9"/>
-      <c r="C119" s="10"/>
+      <c r="A119" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C119" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="8"/>
-      <c r="B120" s="9"/>
-      <c r="C120" s="10"/>
+      <c r="A120" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C120" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="8"/>
-      <c r="B121" s="9"/>
-      <c r="C121" s="10"/>
+      <c r="A121" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C121" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="8"/>
-      <c r="B122" s="9"/>
-      <c r="C122" s="10"/>
+      <c r="A122" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C122" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="8"/>
-      <c r="B123" s="9"/>
-      <c r="C123" s="10"/>
+      <c r="A123" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="8"/>
-      <c r="B124" s="9"/>
-      <c r="C124" s="10"/>
+      <c r="A124" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="8"/>
-      <c r="B125" s="9"/>
-      <c r="C125" s="10"/>
+      <c r="A125" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="8"/>
-      <c r="B126" s="9"/>
-      <c r="C126" s="10"/>
+      <c r="A126" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C126" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="8"/>
-      <c r="B127" s="9"/>
-      <c r="C127" s="10"/>
+      <c r="A127" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C127" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="8"/>
-      <c r="B128" s="9"/>
-      <c r="C128" s="10"/>
+      <c r="A128" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C128" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="8"/>
-      <c r="B129" s="9"/>
-      <c r="C129" s="10"/>
+      <c r="A129" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C129" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="8"/>
-      <c r="B130" s="9"/>
-      <c r="C130" s="10"/>
+      <c r="A130" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B130" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C130" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="8"/>
-      <c r="B131" s="9"/>
-      <c r="C131" s="10"/>
+      <c r="A131" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C131" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="8"/>
-      <c r="B132" s="9"/>
-      <c r="C132" s="10"/>
+      <c r="A132" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C132" s="9" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="8"/>
-      <c r="B133" s="9"/>
-      <c r="C133" s="10"/>
+      <c r="A133" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C133" s="9" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="8"/>
-      <c r="B134" s="9"/>
-      <c r="C134" s="10"/>
+      <c r="A134" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C134" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="8"/>
-      <c r="B135" s="9"/>
-      <c r="C135" s="10"/>
+      <c r="A135" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C135" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="6"/>
-      <c r="B136" s="4"/>
-      <c r="C136" s="6"/>
+      <c r="A136" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C136" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="6"/>
-      <c r="B137" s="4"/>
-      <c r="C137" s="6"/>
+      <c r="A137" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C137" s="9" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="6"/>
-      <c r="B138" s="4"/>
-      <c r="C138" s="6"/>
+      <c r="A138" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="6"/>
-      <c r="B139" s="4"/>
-      <c r="C139" s="6"/>
+      <c r="A139" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" s="6"/>
-      <c r="B140" s="4"/>
-      <c r="C140" s="6"/>
+      <c r="A140" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" s="6"/>
-      <c r="B141" s="4"/>
-      <c r="C141" s="6"/>
+      <c r="A141" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" s="6"/>
-      <c r="B142" s="4"/>
-      <c r="C142" s="6"/>
+      <c r="A142" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="6"/>
-      <c r="B143" s="4"/>
-      <c r="C143" s="6"/>
+      <c r="A143" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="6"/>
-      <c r="B144" s="4"/>
-      <c r="C144" s="6"/>
+      <c r="A144" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="6"/>
-      <c r="B145" s="4"/>
-      <c r="C145" s="6"/>
+      <c r="A145" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="6"/>
-      <c r="B146" s="4"/>
-      <c r="C146" s="6"/>
+      <c r="A146" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" s="6"/>
-      <c r="B147" s="4"/>
-      <c r="C147" s="6"/>
+      <c r="A147" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="148">
-      <c r="A148" s="10"/>
-      <c r="B148" s="9"/>
-      <c r="C148" s="10"/>
+      <c r="A148" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" s="10"/>
-      <c r="B149" s="9"/>
-      <c r="C149" s="10"/>
+      <c r="A149" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="10"/>
-      <c r="B150" s="9"/>
-      <c r="C150" s="10"/>
+      <c r="A150" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C150" s="9" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="10"/>
-      <c r="B151" s="9"/>
-      <c r="C151" s="10"/>
+      <c r="A151" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C151" s="9" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" s="10"/>
-      <c r="B152" s="9"/>
-      <c r="C152" s="10"/>
+      <c r="A152" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C152" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="10"/>
-      <c r="B153" s="9"/>
-      <c r="C153" s="10"/>
+      <c r="A153" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C153" s="9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" s="10"/>
-      <c r="B154" s="9"/>
-      <c r="C154" s="10"/>
+      <c r="A154" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C154" s="9" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="10"/>
-      <c r="B155" s="9"/>
-      <c r="C155" s="10"/>
+      <c r="A155" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C155" s="9" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" s="10"/>
-      <c r="B156" s="9"/>
-      <c r="C156" s="10"/>
+      <c r="A156" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C156" s="9" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="6"/>
-      <c r="B157" s="4"/>
-      <c r="C157" s="6"/>
+      <c r="A157" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C157" s="9" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" s="6"/>
-      <c r="B158" s="4"/>
-      <c r="C158" s="6"/>
+      <c r="A158" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C158" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="6"/>
-      <c r="B159" s="4"/>
-      <c r="C159" s="6"/>
+      <c r="A159" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="6"/>
-      <c r="B160" s="4"/>
-      <c r="C160" s="6"/>
+      <c r="A160" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B160" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" s="6"/>
-      <c r="B161" s="11"/>
-      <c r="C161" s="6"/>
+      <c r="A161" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="162">
-      <c r="A162" s="6"/>
-      <c r="B162" s="11"/>
-      <c r="C162" s="6"/>
+      <c r="A162" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="163">
-      <c r="A163" s="6"/>
-      <c r="B163" s="11"/>
-      <c r="C163" s="6"/>
+      <c r="A163" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" s="6"/>
-      <c r="B164" s="11"/>
+      <c r="A164" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>154</v>
+      </c>
       <c r="C164" s="6"/>
     </row>
     <row r="165">
-      <c r="A165" s="6"/>
-      <c r="B165" s="11"/>
+      <c r="A165" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="C165" s="6"/>
     </row>
     <row r="166">
-      <c r="A166" s="6"/>
-      <c r="B166" s="11"/>
+      <c r="A166" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="C166" s="6"/>
     </row>
     <row r="167">
-      <c r="A167" s="6"/>
-      <c r="B167" s="11"/>
+      <c r="A167" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>157</v>
+      </c>
       <c r="C167" s="6"/>
     </row>
     <row r="168">
-      <c r="A168" s="6"/>
-      <c r="B168" s="11"/>
+      <c r="A168" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B168" s="7" t="s">
+        <v>158</v>
+      </c>
       <c r="C168" s="6"/>
     </row>
     <row r="169">
-      <c r="A169" s="6"/>
-      <c r="B169" s="11"/>
+      <c r="A169" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>159</v>
+      </c>
       <c r="C169" s="6"/>
     </row>
     <row r="170">
-      <c r="A170" s="6"/>
-      <c r="B170" s="11"/>
+      <c r="A170" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>160</v>
+      </c>
       <c r="C170" s="6"/>
     </row>
     <row r="171">
-      <c r="A171" s="6"/>
-      <c r="B171" s="11"/>
-      <c r="C171" s="6"/>
+      <c r="A171" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C171" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="172">
-      <c r="A172" s="6"/>
-      <c r="B172" s="11"/>
+      <c r="A172" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="C172" s="6"/>
     </row>
     <row r="173">
-      <c r="A173" s="6"/>
-      <c r="B173" s="11"/>
+      <c r="A173" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="C173" s="6"/>
     </row>
     <row r="174">
-      <c r="A174" s="6"/>
-      <c r="B174" s="11"/>
+      <c r="A174" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>162</v>
+      </c>
       <c r="C174" s="6"/>
     </row>
     <row r="175">
-      <c r="A175" s="6"/>
-      <c r="B175" s="11"/>
+      <c r="A175" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>163</v>
+      </c>
       <c r="C175" s="6"/>
     </row>
     <row r="176">
-      <c r="A176" s="6"/>
-      <c r="B176" s="11"/>
+      <c r="A176" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B176" s="4" t="s">
+        <v>164</v>
+      </c>
       <c r="C176" s="6"/>
     </row>
     <row r="177">
-      <c r="A177" s="6"/>
-      <c r="B177" s="11"/>
+      <c r="A177" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>165</v>
+      </c>
       <c r="C177" s="6"/>
     </row>
     <row r="178">
-      <c r="A178" s="6"/>
-      <c r="B178" s="11"/>
+      <c r="A178" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="C178" s="6"/>
     </row>
     <row r="179">
-      <c r="A179" s="6"/>
-      <c r="B179" s="11"/>
+      <c r="A179" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>166</v>
+      </c>
       <c r="C179" s="6"/>
     </row>
     <row r="180">
-      <c r="A180" s="6"/>
-      <c r="B180" s="11"/>
-      <c r="C180" s="6"/>
+      <c r="A180" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="181">
-      <c r="A181" s="6"/>
-      <c r="B181" s="11"/>
-      <c r="C181" s="6"/>
+      <c r="A181" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B181" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" s="6"/>
-      <c r="B182" s="11"/>
-      <c r="C182" s="6"/>
+      <c r="A182" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="183">
-      <c r="A183" s="6"/>
-      <c r="B183" s="11"/>
-      <c r="C183" s="6"/>
+      <c r="A183" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="184">
-      <c r="A184" s="6"/>
-      <c r="B184" s="11"/>
-      <c r="C184" s="6"/>
+      <c r="A184" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" s="6"/>
-      <c r="B185" s="11"/>
-      <c r="C185" s="6"/>
+      <c r="A185" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="186">
-      <c r="A186" s="6"/>
-      <c r="B186" s="11"/>
-      <c r="C186" s="6"/>
+      <c r="A186" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="187">
-      <c r="A187" s="6"/>
-      <c r="B187" s="11"/>
-      <c r="C187" s="6"/>
+      <c r="A187" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C187" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="188">
-      <c r="A188" s="6"/>
-      <c r="B188" s="11"/>
-      <c r="C188" s="6"/>
+      <c r="A188" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B188" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="189">
-      <c r="A189" s="6"/>
-      <c r="B189" s="11"/>
+      <c r="A189" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>174</v>
+      </c>
       <c r="C189" s="6"/>
     </row>
     <row r="190">
@@ -5971,18 +7096,35 @@
       <c r="B1037" s="11"/>
       <c r="C1037" s="6"/>
     </row>
+    <row r="1038">
+      <c r="A1038" s="6"/>
+      <c r="B1038" s="11"/>
+      <c r="C1038" s="6"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="6"/>
+      <c r="B1039" s="11"/>
+      <c r="C1039" s="6"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A1037">
-      <formula1>"girton-wadsworth,yale-wadsworth,morrison-wadsworth,evans-wadsworth,jewell-garrison,alameda-wadsworth,1st-wadsworth,2nd-union,bowles-coalmine,colfax-simms,colfax-kipling,colfax-wadsworth,colfax-sheridan,mississippi-wadsworth,25th-sheridan,24th-sheridan,spe"&amp;"er-federal"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C1:C4 C9:C1039">
+      <formula1>"storefront_main,t-shirt,street_sign,advertisement,storefront_accessory,car_signs,instructions,code_type,grafitti,other,truck,lot_sign,other_sign,bus"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C1:C1037">
-      <formula1>"storefront_main,t-shirt,street_sign,advertisement,storefront_accessory,car_signs,instructions,code_type,grafitti,other"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A4 A9:A1039">
+      <formula1>"girton-wadsworth,yale-wadsworth,morrison-wadsworth,evans-wadsworth,jewell-garrison,alameda-wadsworth,1st-wadsworth,2nd-union,bowles-coalmine,colfax-simms,colfax-kipling,colfax-wadsworth,colfax-sheridan,mississippi-wadsworth,25th-sheridan,24th-sheridan,spe"&amp;"er-federal,mississippi-sheridan"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B21"/>
+    <hyperlink r:id="rId1" ref="B52"/>
+    <hyperlink r:id="rId2" ref="B67"/>
+    <hyperlink r:id="rId3" ref="B100"/>
+    <hyperlink r:id="rId4" ref="B111"/>
+    <hyperlink r:id="rId5" ref="B113"/>
+    <hyperlink r:id="rId6" ref="B130"/>
+    <hyperlink r:id="rId7" ref="B168"/>
+    <hyperlink r:id="rId8" ref="B181"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>